<commit_message>
fixed bug creatied students by resolve does not have any name
</commit_message>
<xml_diff>
--- a/docs/data/sample2.xlsx
+++ b/docs/data/sample2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\erenimo\projects\ses\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\erenimo\projects\ses\docs\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB4E4CCD-090D-4AEE-BFF2-AE5F6BDECD86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31C2EBB2-EA34-4B2F-9355-8EBF42DA2B09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -212,9 +212,6 @@
     <t>studentname24</t>
   </si>
   <si>
-    <t>studentname25</t>
-  </si>
-  <si>
     <t>studentsurname1</t>
   </si>
   <si>
@@ -287,9 +284,6 @@
     <t>studentsurname24</t>
   </si>
   <si>
-    <t>studentsurname25</t>
-  </si>
-  <si>
     <t>Project(%10)_0833AB</t>
   </si>
   <si>
@@ -366,6 +360,12 @@
   </si>
   <si>
     <t>221400050</t>
+  </si>
+  <si>
+    <t>asd</t>
+  </si>
+  <si>
+    <t>fgh</t>
   </si>
 </sst>
 </file>
@@ -1705,7 +1705,7 @@
         <v>33</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="J1" s="3" t="s">
         <v>34</v>
@@ -1719,13 +1719,13 @@
         <v>7</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>35</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>8</v>
@@ -1734,20 +1734,20 @@
         <v>7</v>
       </c>
       <c r="G2" s="9">
-        <f t="shared" ref="G2:H50" ca="1" si="0">TRUNC(60 + ((RAND()*100 - 0) * (100 - 60) / (100 - 0)))</f>
-        <v>85</v>
+        <f ca="1">TRUNC(30 + ((RAND()*100 - 0) * (100 - 60) / (100 - 0)))</f>
+        <v>59</v>
       </c>
       <c r="H2" s="9">
-        <f ca="1">TRUNC(60 + ((RAND()*100 - 0) * (100 - 60) / (100 - 0)))</f>
-        <v>68</v>
+        <f t="shared" ref="H2:J17" ca="1" si="0">TRUNC(30 + ((RAND()*100 - 0) * (100 - 60) / (100 - 0)))</f>
+        <v>35</v>
       </c>
       <c r="I2" s="9">
-        <f ca="1">TRUNC(30 + ((RAND()*100 - 0) * (60 - 30) / (100 - 0)))</f>
-        <v>34</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>53</v>
       </c>
       <c r="J2" s="9">
-        <f ca="1">TRUNC(30 + ((RAND()*100 - 0) * (60 - 30) / (100 - 0)))</f>
-        <v>31</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>54</v>
       </c>
       <c r="K2" s="6"/>
     </row>
@@ -1756,13 +1756,13 @@
         <v>9</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>36</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E3" s="7" t="s">
         <v>8</v>
@@ -1771,20 +1771,16 @@
         <v>7</v>
       </c>
       <c r="G3" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="H3" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>62</v>
+        <v>10</v>
       </c>
       <c r="I3" s="9">
-        <f t="shared" ref="I3:J50" ca="1" si="1">TRUNC(30 + ((RAND()*100 - 0) * (60 - 30) / (100 - 0)))</f>
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="J3" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="K3" s="8"/>
     </row>
@@ -1793,13 +1789,13 @@
         <v>10</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>37</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>10</v>
@@ -1808,20 +1804,20 @@
         <v>7</v>
       </c>
       <c r="G4" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>79</v>
+        <f t="shared" ref="G3:J26" ca="1" si="1">TRUNC(30 + ((RAND()*100 - 0) * (100 - 60) / (100 - 0)))</f>
+        <v>34</v>
       </c>
       <c r="H4" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="I4" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>59</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>49</v>
       </c>
       <c r="J4" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>40</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>31</v>
       </c>
       <c r="K4" s="8"/>
     </row>
@@ -1830,13 +1826,13 @@
         <v>8</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>38</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>10</v>
@@ -1845,20 +1841,20 @@
         <v>7</v>
       </c>
       <c r="G5" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>94</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>62</v>
       </c>
       <c r="H5" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>89</v>
+        <v>59</v>
       </c>
       <c r="I5" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>64</v>
       </c>
       <c r="J5" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>57</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>37</v>
       </c>
       <c r="K5" s="8"/>
     </row>
@@ -1867,13 +1863,13 @@
         <v>11</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>39</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>8</v>
@@ -1882,20 +1878,20 @@
         <v>7</v>
       </c>
       <c r="G6" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>79</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>51</v>
       </c>
       <c r="H6" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>91</v>
+        <v>54</v>
       </c>
       <c r="I6" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>59</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>37</v>
       </c>
       <c r="J6" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>57</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>65</v>
       </c>
       <c r="K6" s="8"/>
     </row>
@@ -1904,13 +1900,13 @@
         <v>12</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>40</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>10</v>
@@ -1919,20 +1915,20 @@
         <v>7</v>
       </c>
       <c r="G7" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>88</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>47</v>
       </c>
       <c r="H7" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="I7" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>44</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>42</v>
       </c>
       <c r="J7" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>45</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>67</v>
       </c>
       <c r="K7" s="8"/>
     </row>
@@ -1941,13 +1937,13 @@
         <v>13</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>41</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>10</v>
@@ -1956,20 +1952,20 @@
         <v>7</v>
       </c>
       <c r="G8" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>94</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>47</v>
       </c>
       <c r="H8" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>99</v>
+        <v>41</v>
       </c>
       <c r="I8" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>49</v>
       </c>
       <c r="J8" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>40</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>33</v>
       </c>
       <c r="K8" s="8"/>
     </row>
@@ -1978,13 +1974,13 @@
         <v>14</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>42</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E9" s="7" t="s">
         <v>10</v>
@@ -1993,20 +1989,20 @@
         <v>7</v>
       </c>
       <c r="G9" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>78</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>50</v>
       </c>
       <c r="H9" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>93</v>
+        <v>63</v>
       </c>
       <c r="I9" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>49</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>42</v>
       </c>
       <c r="J9" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>33</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>67</v>
       </c>
       <c r="K9" s="8"/>
     </row>
@@ -2015,13 +2011,13 @@
         <v>15</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>43</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E10" s="7" t="s">
         <v>10</v>
@@ -2030,20 +2026,20 @@
         <v>7</v>
       </c>
       <c r="G10" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>74</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>31</v>
       </c>
       <c r="H10" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="I10" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>68</v>
       </c>
       <c r="J10" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>39</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>49</v>
       </c>
       <c r="K10" s="8"/>
     </row>
@@ -2052,13 +2048,13 @@
         <v>16</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>44</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>10</v>
@@ -2067,20 +2063,20 @@
         <v>7</v>
       </c>
       <c r="G11" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>84</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>34</v>
       </c>
       <c r="H11" s="9">
         <f t="shared" ca="1" si="0"/>
         <v>61</v>
       </c>
       <c r="I11" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>51</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45</v>
       </c>
       <c r="J11" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>43</v>
       </c>
       <c r="K11" s="8"/>
     </row>
@@ -2089,13 +2085,13 @@
         <v>17</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>45</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E12" s="7" t="s">
         <v>10</v>
@@ -2104,20 +2100,20 @@
         <v>7</v>
       </c>
       <c r="G12" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>95</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>68</v>
       </c>
       <c r="H12" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="I12" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>57</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>62</v>
       </c>
       <c r="J12" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>56</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45</v>
       </c>
       <c r="K12" s="8"/>
     </row>
@@ -2126,13 +2122,13 @@
         <v>18</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>46</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E13" s="7" t="s">
         <v>10</v>
@@ -2141,20 +2137,20 @@
         <v>7</v>
       </c>
       <c r="G13" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>71</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>38</v>
       </c>
       <c r="H13" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>71</v>
+        <v>31</v>
       </c>
       <c r="I13" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>42</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>49</v>
       </c>
       <c r="J13" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>41</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>65</v>
       </c>
       <c r="K13" s="8"/>
     </row>
@@ -2163,13 +2159,13 @@
         <v>19</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>47</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>10</v>
@@ -2178,20 +2174,20 @@
         <v>7</v>
       </c>
       <c r="G14" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>89</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>53</v>
       </c>
       <c r="H14" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="I14" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>40</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>50</v>
       </c>
       <c r="J14" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>53</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>50</v>
       </c>
       <c r="K14" s="8"/>
     </row>
@@ -2200,13 +2196,13 @@
         <v>20</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>48</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E15" s="7" t="s">
         <v>10</v>
@@ -2215,20 +2211,20 @@
         <v>7</v>
       </c>
       <c r="G15" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>99</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>38</v>
       </c>
       <c r="H15" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>95</v>
+        <v>46</v>
       </c>
       <c r="I15" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>45</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>40</v>
       </c>
       <c r="J15" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>42</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>67</v>
       </c>
       <c r="K15" s="8"/>
     </row>
@@ -2237,13 +2233,13 @@
         <v>21</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>49</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>10</v>
@@ -2252,20 +2248,20 @@
         <v>7</v>
       </c>
       <c r="G16" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>99</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>54</v>
       </c>
       <c r="H16" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>95</v>
+        <v>54</v>
       </c>
       <c r="I16" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>42</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>48</v>
       </c>
       <c r="J16" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>47</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>53</v>
       </c>
       <c r="K16" s="8"/>
     </row>
@@ -2274,13 +2270,13 @@
         <v>22</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>50</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>10</v>
@@ -2289,20 +2285,20 @@
         <v>7</v>
       </c>
       <c r="G17" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>97</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>65</v>
       </c>
       <c r="H17" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>68</v>
+        <v>43</v>
       </c>
       <c r="I17" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>48</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>59</v>
       </c>
       <c r="J17" s="9">
-        <f t="shared" ca="1" si="1"/>
-        <v>48</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>38</v>
       </c>
       <c r="K17" s="8"/>
     </row>
@@ -2311,13 +2307,13 @@
         <v>23</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>51</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E18" s="7" t="s">
         <v>8</v>
@@ -2326,20 +2322,20 @@
         <v>7</v>
       </c>
       <c r="G18" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>73</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>50</v>
       </c>
       <c r="H18" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>94</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>61</v>
       </c>
       <c r="I18" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J18" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="K18" s="8"/>
     </row>
@@ -2348,13 +2344,13 @@
         <v>24</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>52</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E19" s="7" t="s">
         <v>10</v>
@@ -2363,20 +2359,20 @@
         <v>7</v>
       </c>
       <c r="G19" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>76</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>39</v>
       </c>
       <c r="H19" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>72</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>69</v>
       </c>
       <c r="I19" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="J19" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>39</v>
+        <v>69</v>
       </c>
       <c r="K19" s="8"/>
     </row>
@@ -2385,13 +2381,13 @@
         <v>25</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>53</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E20" s="7" t="s">
         <v>10</v>
@@ -2400,20 +2396,20 @@
         <v>7</v>
       </c>
       <c r="G20" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>94</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>48</v>
       </c>
       <c r="H20" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>61</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>31</v>
       </c>
       <c r="I20" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="J20" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="K20" s="8"/>
     </row>
@@ -2422,13 +2418,13 @@
         <v>26</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>54</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E21" s="7" t="s">
         <v>10</v>
@@ -2437,20 +2433,20 @@
         <v>7</v>
       </c>
       <c r="G21" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>84</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>34</v>
       </c>
       <c r="H21" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>84</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>32</v>
       </c>
       <c r="I21" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="J21" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="K21" s="8"/>
     </row>
@@ -2459,13 +2455,13 @@
         <v>27</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>55</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E22" s="7" t="s">
         <v>8</v>
@@ -2474,20 +2470,20 @@
         <v>7</v>
       </c>
       <c r="G22" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>65</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46</v>
       </c>
       <c r="H22" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>94</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>33</v>
       </c>
       <c r="I22" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="J22" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="K22" s="8"/>
     </row>
@@ -2496,13 +2492,13 @@
         <v>28</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>56</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E23" s="7" t="s">
         <v>10</v>
@@ -2511,20 +2507,20 @@
         <v>7</v>
       </c>
       <c r="G23" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>90</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>54</v>
       </c>
       <c r="H23" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>82</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>49</v>
       </c>
       <c r="I23" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="J23" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="K23" s="8"/>
     </row>
@@ -2533,13 +2529,13 @@
         <v>29</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>10</v>
@@ -2548,20 +2544,20 @@
         <v>7</v>
       </c>
       <c r="G24" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>85</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45</v>
       </c>
       <c r="H24" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>92</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>63</v>
       </c>
       <c r="I24" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="J24" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>42</v>
+        <v>66</v>
       </c>
       <c r="K24" s="8"/>
     </row>
@@ -2570,13 +2566,13 @@
         <v>30</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>58</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>10</v>
@@ -2585,20 +2581,20 @@
         <v>7</v>
       </c>
       <c r="G25" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>85</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>66</v>
       </c>
       <c r="H25" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>91</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45</v>
       </c>
       <c r="I25" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="J25" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K25" s="8"/>
     </row>
@@ -2607,13 +2603,13 @@
         <v>31</v>
       </c>
       <c r="B26" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="D26" s="5" t="s">
         <v>110</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>84</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>10</v>
@@ -2622,20 +2618,20 @@
         <v>7</v>
       </c>
       <c r="G26" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>84</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>33</v>
       </c>
       <c r="H26" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>93</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>54</v>
       </c>
       <c r="I26" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="J26" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="K26" s="8"/>
     </row>

</xml_diff>